<commit_message>
planner docker file is changed
</commit_message>
<xml_diff>
--- a/backend-Planner/plannerAgentBackend/uploaded_excels/planner_agent_data_nushan.xlsx
+++ b/backend-Planner/plannerAgentBackend/uploaded_excels/planner_agent_data_nushan.xlsx
@@ -5,11 +5,11 @@
   <workbookPr defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\7th\FinalYearProject\dataset\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eanus\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12315" firstSheet="2" activeTab="5"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12315" firstSheet="2" activeTab="12"/>
   </bookViews>
   <sheets>
     <sheet name="Semester 1" sheetId="1" r:id="rId1"/>
@@ -18,12 +18,14 @@
     <sheet name="Semester 4" sheetId="4" r:id="rId4"/>
     <sheet name="Semester 5" sheetId="5" r:id="rId5"/>
     <sheet name="module codes" sheetId="6" r:id="rId6"/>
-    <sheet name="Sheet6" sheetId="13" r:id="rId7"/>
-    <sheet name="Sheet5" sheetId="12" r:id="rId8"/>
-    <sheet name="module codes2" sheetId="8" r:id="rId9"/>
-    <sheet name="Sheet2" sheetId="10" r:id="rId10"/>
-    <sheet name="Sheet4" sheetId="11" r:id="rId11"/>
-    <sheet name="halls" sheetId="7" r:id="rId12"/>
+    <sheet name="halls2" sheetId="14" r:id="rId7"/>
+    <sheet name="Sheet6" sheetId="13" r:id="rId8"/>
+    <sheet name="Sheet5" sheetId="12" r:id="rId9"/>
+    <sheet name="module codes2" sheetId="8" r:id="rId10"/>
+    <sheet name="Sheet2" sheetId="10" r:id="rId11"/>
+    <sheet name="Sheet4" sheetId="11" r:id="rId12"/>
+    <sheet name="halls" sheetId="7" r:id="rId13"/>
+    <sheet name="halls-exam" sheetId="15" r:id="rId14"/>
   </sheets>
   <calcPr calcId="152511"/>
   <extLst>
@@ -35,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7801" uniqueCount="1323">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7917" uniqueCount="1325">
   <si>
     <t>Hall</t>
   </si>
@@ -4004,6 +4006,12 @@
   </si>
   <si>
     <t>IS8201: Day=Sun, Hall=AUD, Slot=4</t>
+  </si>
+  <si>
+    <t>GYM</t>
+  </si>
+  <si>
+    <t>Gym</t>
   </si>
 </sst>
 </file>
@@ -7866,6 +7874,284 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:G10"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="7" max="7" width="23" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7">
+      <c r="A1" t="s">
+        <v>589</v>
+      </c>
+      <c r="B1" t="s">
+        <v>590</v>
+      </c>
+      <c r="C1" t="s">
+        <v>591</v>
+      </c>
+      <c r="D1" t="s">
+        <v>592</v>
+      </c>
+      <c r="E1" t="s">
+        <v>593</v>
+      </c>
+      <c r="F1" t="s">
+        <v>594</v>
+      </c>
+      <c r="G1" t="s">
+        <v>632</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2" t="str">
+        <f>IF(MID(A2,3,1)=" ",LEFT(A2,2)&amp;MID(A2,4,LEN(A2)-3),A2)</f>
+        <v>CE1202</v>
+      </c>
+      <c r="D2" t="str">
+        <f>MID(C2,4,1)</f>
+        <v>2</v>
+      </c>
+      <c r="E2" t="b">
+        <f>IF(F2="IS",TRUE,FALSE)</f>
+        <v>0</v>
+      </c>
+      <c r="F2" t="str">
+        <f>LEFT(C2,2)</f>
+        <v>CE</v>
+      </c>
+      <c r="G2">
+        <v>550</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7">
+      <c r="A3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3" t="str">
+        <f t="shared" ref="C3:C10" si="0">IF(MID(A3,3,1)=" ",LEFT(A3,2)&amp;MID(A3,4,LEN(A3)-3),A3)</f>
+        <v>CE1101</v>
+      </c>
+      <c r="D3" t="str">
+        <f t="shared" ref="D3:D9" si="1">MID(C3,4,1)</f>
+        <v>1</v>
+      </c>
+      <c r="E3" t="b">
+        <f t="shared" ref="E3:E10" si="2">IF(F3="IS",TRUE,FALSE)</f>
+        <v>0</v>
+      </c>
+      <c r="F3" t="str">
+        <f t="shared" ref="F3:F10" si="3">LEFT(C3,2)</f>
+        <v>CE</v>
+      </c>
+      <c r="G3">
+        <v>550</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4">
+        <v>1</v>
+      </c>
+      <c r="C4" t="str">
+        <f t="shared" si="0"/>
+        <v>EE1301</v>
+      </c>
+      <c r="D4" t="str">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
+      <c r="E4" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="F4" t="str">
+        <f t="shared" si="3"/>
+        <v>EE</v>
+      </c>
+      <c r="G4">
+        <v>550</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7">
+      <c r="A5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5">
+        <v>1</v>
+      </c>
+      <c r="C5" t="str">
+        <f t="shared" si="0"/>
+        <v>EE1101</v>
+      </c>
+      <c r="D5" t="str">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="E5" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="F5" t="str">
+        <f t="shared" si="3"/>
+        <v>EE</v>
+      </c>
+      <c r="G5">
+        <v>550</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
+      <c r="A6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6">
+        <v>1</v>
+      </c>
+      <c r="C6" t="str">
+        <f t="shared" si="0"/>
+        <v>ME1201</v>
+      </c>
+      <c r="D6" t="str">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="E6" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="F6" t="str">
+        <f t="shared" si="3"/>
+        <v>ME</v>
+      </c>
+      <c r="G6">
+        <v>550</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7">
+      <c r="A7" t="s">
+        <v>16</v>
+      </c>
+      <c r="B7">
+        <v>1</v>
+      </c>
+      <c r="C7" t="str">
+        <f t="shared" si="0"/>
+        <v>ME1202</v>
+      </c>
+      <c r="D7" t="str">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="E7" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="F7" t="str">
+        <f t="shared" si="3"/>
+        <v>ME</v>
+      </c>
+      <c r="G7">
+        <v>550</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7">
+      <c r="A8" t="s">
+        <v>18</v>
+      </c>
+      <c r="B8">
+        <v>1</v>
+      </c>
+      <c r="C8" t="str">
+        <f t="shared" si="0"/>
+        <v>IS1402</v>
+      </c>
+      <c r="D8" t="str">
+        <f t="shared" si="1"/>
+        <v>4</v>
+      </c>
+      <c r="E8" t="b">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="F8" t="str">
+        <f t="shared" si="3"/>
+        <v>IS</v>
+      </c>
+      <c r="G8">
+        <v>550</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7">
+      <c r="A9" t="s">
+        <v>20</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9" t="str">
+        <f t="shared" si="0"/>
+        <v>IS1301</v>
+      </c>
+      <c r="D9" t="str">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
+      <c r="E9" t="b">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="F9" t="str">
+        <f t="shared" si="3"/>
+        <v>IS</v>
+      </c>
+      <c r="G9">
+        <v>550</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7">
+      <c r="A10" t="s">
+        <v>22</v>
+      </c>
+      <c r="B10">
+        <v>1</v>
+      </c>
+      <c r="C10" t="str">
+        <f t="shared" si="0"/>
+        <v>IS1003</v>
+      </c>
+      <c r="D10">
+        <v>2</v>
+      </c>
+      <c r="E10" t="b">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="F10" t="str">
+        <f t="shared" si="3"/>
+        <v>IS</v>
+      </c>
+      <c r="G10">
+        <v>550</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:G100"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -10778,7 +11064,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:B248"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -12776,7 +13062,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H26"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -13055,6 +13341,289 @@
         <v>572</v>
       </c>
     </row>
+    <row r="25" spans="1:1">
+      <c r="A25" s="33"/>
+    </row>
+    <row r="26" spans="1:1">
+      <c r="A26" s="33"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:H17"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="34.140625" customWidth="1"/>
+    <col min="5" max="5" width="21.28515625" customWidth="1"/>
+    <col min="6" max="6" width="21.7109375" customWidth="1"/>
+    <col min="7" max="7" width="31" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8">
+      <c r="A1" t="s">
+        <v>594</v>
+      </c>
+      <c r="B1" t="s">
+        <v>596</v>
+      </c>
+      <c r="C1" t="s">
+        <v>597</v>
+      </c>
+      <c r="D1" t="s">
+        <v>598</v>
+      </c>
+      <c r="E1" t="s">
+        <v>599</v>
+      </c>
+      <c r="F1" t="s">
+        <v>600</v>
+      </c>
+      <c r="G1" t="s">
+        <v>601</v>
+      </c>
+      <c r="H1" t="s">
+        <v>595</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8">
+      <c r="A2" t="s">
+        <v>631</v>
+      </c>
+      <c r="B2">
+        <v>16</v>
+      </c>
+      <c r="C2">
+        <v>0</v>
+      </c>
+      <c r="D2">
+        <v>2</v>
+      </c>
+      <c r="E2" t="s">
+        <v>173</v>
+      </c>
+      <c r="F2" t="s">
+        <v>173</v>
+      </c>
+      <c r="G2" t="s">
+        <v>602</v>
+      </c>
+      <c r="H2">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8">
+      <c r="A3" t="s">
+        <v>631</v>
+      </c>
+      <c r="B3">
+        <v>17</v>
+      </c>
+      <c r="C3">
+        <v>0</v>
+      </c>
+      <c r="D3">
+        <v>2</v>
+      </c>
+      <c r="E3" t="s">
+        <v>79</v>
+      </c>
+      <c r="F3" t="s">
+        <v>79</v>
+      </c>
+      <c r="G3" t="s">
+        <v>603</v>
+      </c>
+      <c r="H3">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8">
+      <c r="A4" t="s">
+        <v>631</v>
+      </c>
+      <c r="B4">
+        <v>18</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+      <c r="D4">
+        <v>2</v>
+      </c>
+      <c r="E4" t="s">
+        <v>110</v>
+      </c>
+      <c r="F4" t="s">
+        <v>110</v>
+      </c>
+      <c r="G4" t="s">
+        <v>604</v>
+      </c>
+      <c r="H4">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8">
+      <c r="A5" t="s">
+        <v>631</v>
+      </c>
+      <c r="B5">
+        <v>19</v>
+      </c>
+      <c r="C5">
+        <v>0</v>
+      </c>
+      <c r="D5">
+        <v>2</v>
+      </c>
+      <c r="E5" t="s">
+        <v>73</v>
+      </c>
+      <c r="F5" t="s">
+        <v>73</v>
+      </c>
+      <c r="G5" t="s">
+        <v>605</v>
+      </c>
+      <c r="H5">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8">
+      <c r="A6" t="s">
+        <v>631</v>
+      </c>
+      <c r="B6">
+        <v>22</v>
+      </c>
+      <c r="C6">
+        <v>0</v>
+      </c>
+      <c r="D6">
+        <v>2</v>
+      </c>
+      <c r="E6" t="s">
+        <v>276</v>
+      </c>
+      <c r="F6" t="s">
+        <v>276</v>
+      </c>
+      <c r="G6" t="s">
+        <v>606</v>
+      </c>
+      <c r="H6">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8">
+      <c r="A7" t="s">
+        <v>631</v>
+      </c>
+      <c r="B7">
+        <v>23</v>
+      </c>
+      <c r="C7">
+        <v>0</v>
+      </c>
+      <c r="D7">
+        <v>2</v>
+      </c>
+      <c r="E7" t="s">
+        <v>99</v>
+      </c>
+      <c r="F7" t="s">
+        <v>99</v>
+      </c>
+      <c r="G7" t="s">
+        <v>607</v>
+      </c>
+      <c r="H7">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8">
+      <c r="A8" t="s">
+        <v>631</v>
+      </c>
+      <c r="B8">
+        <v>24</v>
+      </c>
+      <c r="C8">
+        <v>0</v>
+      </c>
+      <c r="D8">
+        <v>2</v>
+      </c>
+      <c r="E8" t="s">
+        <v>251</v>
+      </c>
+      <c r="F8" t="s">
+        <v>251</v>
+      </c>
+      <c r="G8" t="s">
+        <v>608</v>
+      </c>
+      <c r="H8">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8">
+      <c r="A9" t="s">
+        <v>631</v>
+      </c>
+      <c r="B9">
+        <v>25</v>
+      </c>
+      <c r="C9">
+        <v>0</v>
+      </c>
+      <c r="D9">
+        <v>2</v>
+      </c>
+      <c r="E9" t="s">
+        <v>100</v>
+      </c>
+      <c r="F9" t="s">
+        <v>100</v>
+      </c>
+      <c r="G9" t="s">
+        <v>609</v>
+      </c>
+      <c r="H9">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8">
+      <c r="A10" t="s">
+        <v>631</v>
+      </c>
+      <c r="B10">
+        <v>47</v>
+      </c>
+      <c r="C10">
+        <v>0</v>
+      </c>
+      <c r="D10">
+        <v>2</v>
+      </c>
+      <c r="E10" t="s">
+        <v>1323</v>
+      </c>
+      <c r="F10" t="s">
+        <v>1323</v>
+      </c>
+      <c r="G10" t="s">
+        <v>1324</v>
+      </c>
+      <c r="H10">
+        <v>340</v>
+      </c>
+    </row>
     <row r="11" spans="1:8">
       <c r="A11" t="s">
         <v>631</v>
@@ -13161,10 +13730,10 @@
     </row>
     <row r="15" spans="1:8">
       <c r="A15" t="s">
-        <v>86</v>
+        <v>631</v>
       </c>
       <c r="B15">
-        <v>31</v>
+        <v>44</v>
       </c>
       <c r="C15">
         <v>0</v>
@@ -13173,24 +13742,24 @@
         <v>2</v>
       </c>
       <c r="E15" t="s">
-        <v>619</v>
+        <v>625</v>
       </c>
       <c r="F15" t="s">
-        <v>619</v>
+        <v>625</v>
       </c>
       <c r="G15" t="s">
-        <v>619</v>
+        <v>626</v>
       </c>
       <c r="H15">
-        <v>75</v>
+        <v>50</v>
       </c>
     </row>
     <row r="16" spans="1:8">
       <c r="A16" t="s">
-        <v>86</v>
+        <v>631</v>
       </c>
       <c r="B16">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="C16">
         <v>0</v>
@@ -13199,24 +13768,24 @@
         <v>2</v>
       </c>
       <c r="E16" t="s">
-        <v>620</v>
+        <v>627</v>
       </c>
       <c r="F16" t="s">
-        <v>620</v>
+        <v>627</v>
       </c>
       <c r="G16" t="s">
-        <v>620</v>
+        <v>628</v>
       </c>
       <c r="H16">
-        <v>125</v>
+        <v>45</v>
       </c>
     </row>
     <row r="17" spans="1:8">
       <c r="A17" t="s">
-        <v>87</v>
+        <v>631</v>
       </c>
       <c r="B17">
-        <v>33</v>
+        <v>46</v>
       </c>
       <c r="C17">
         <v>0</v>
@@ -13225,206 +13794,20 @@
         <v>2</v>
       </c>
       <c r="E17" t="s">
-        <v>621</v>
+        <v>629</v>
       </c>
       <c r="F17" t="s">
-        <v>621</v>
+        <v>629</v>
       </c>
       <c r="G17" t="s">
-        <v>621</v>
+        <v>630</v>
       </c>
       <c r="H17">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8">
-      <c r="A18" t="s">
-        <v>87</v>
-      </c>
-      <c r="B18">
-        <v>34</v>
-      </c>
-      <c r="C18">
-        <v>0</v>
-      </c>
-      <c r="D18">
-        <v>2</v>
-      </c>
-      <c r="E18" t="s">
-        <v>622</v>
-      </c>
-      <c r="F18" t="s">
-        <v>622</v>
-      </c>
-      <c r="G18" t="s">
-        <v>622</v>
-      </c>
-      <c r="H18">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8">
-      <c r="A19" t="s">
-        <v>155</v>
-      </c>
-      <c r="B19">
-        <v>35</v>
-      </c>
-      <c r="C19">
-        <v>0</v>
-      </c>
-      <c r="D19">
-        <v>2</v>
-      </c>
-      <c r="E19" t="s">
-        <v>623</v>
-      </c>
-      <c r="F19" t="s">
-        <v>623</v>
-      </c>
-      <c r="G19" t="s">
-        <v>623</v>
-      </c>
-      <c r="H19">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8">
-      <c r="A20" t="s">
-        <v>155</v>
-      </c>
-      <c r="B20">
-        <v>36</v>
-      </c>
-      <c r="C20">
-        <v>0</v>
-      </c>
-      <c r="D20">
-        <v>2</v>
-      </c>
-      <c r="E20" t="s">
-        <v>624</v>
-      </c>
-      <c r="F20" t="s">
-        <v>624</v>
-      </c>
-      <c r="G20" t="s">
-        <v>624</v>
-      </c>
-      <c r="H20">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8">
-      <c r="A21" t="s">
-        <v>631</v>
-      </c>
-      <c r="B21">
-        <v>43</v>
-      </c>
-      <c r="C21">
-        <v>0</v>
-      </c>
-      <c r="D21">
-        <v>5</v>
-      </c>
-      <c r="E21" t="s">
-        <v>625</v>
-      </c>
-      <c r="F21" t="s">
-        <v>625</v>
-      </c>
-      <c r="H21">
         <v>50</v>
       </c>
-    </row>
-    <row r="22" spans="1:8">
-      <c r="A22" t="s">
-        <v>631</v>
-      </c>
-      <c r="B22">
-        <v>44</v>
-      </c>
-      <c r="C22">
-        <v>0</v>
-      </c>
-      <c r="D22">
-        <v>2</v>
-      </c>
-      <c r="E22" t="s">
-        <v>625</v>
-      </c>
-      <c r="F22" t="s">
-        <v>625</v>
-      </c>
-      <c r="G22" t="s">
-        <v>626</v>
-      </c>
-      <c r="H22">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8">
-      <c r="A23" t="s">
-        <v>631</v>
-      </c>
-      <c r="B23">
-        <v>45</v>
-      </c>
-      <c r="C23">
-        <v>0</v>
-      </c>
-      <c r="D23">
-        <v>2</v>
-      </c>
-      <c r="E23" t="s">
-        <v>627</v>
-      </c>
-      <c r="F23" t="s">
-        <v>627</v>
-      </c>
-      <c r="G23" t="s">
-        <v>628</v>
-      </c>
-      <c r="H23">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8">
-      <c r="A24" t="s">
-        <v>631</v>
-      </c>
-      <c r="B24">
-        <v>46</v>
-      </c>
-      <c r="C24">
-        <v>0</v>
-      </c>
-      <c r="D24">
-        <v>2</v>
-      </c>
-      <c r="E24" t="s">
-        <v>629</v>
-      </c>
-      <c r="F24" t="s">
-        <v>629</v>
-      </c>
-      <c r="G24" t="s">
-        <v>630</v>
-      </c>
-      <c r="H24">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="25" spans="1:8">
-      <c r="A25" s="33"/>
-    </row>
-    <row r="26" spans="1:8">
-      <c r="A26" s="33"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -41607,7 +41990,7 @@
         <v>ME5305</v>
       </c>
       <c r="D67">
-        <f t="shared" ref="D67:D80" si="5">VALUE(MID(C67,4,1))</f>
+        <f t="shared" ref="D67:D77" si="5">VALUE(MID(C67,4,1))</f>
         <v>3</v>
       </c>
       <c r="E67" t="b">
@@ -42569,6 +42952,640 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:H24"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="86.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8">
+      <c r="A1" t="s">
+        <v>594</v>
+      </c>
+      <c r="B1" t="s">
+        <v>596</v>
+      </c>
+      <c r="C1" t="s">
+        <v>597</v>
+      </c>
+      <c r="D1" t="s">
+        <v>598</v>
+      </c>
+      <c r="E1" t="s">
+        <v>599</v>
+      </c>
+      <c r="F1" t="s">
+        <v>600</v>
+      </c>
+      <c r="G1" t="s">
+        <v>601</v>
+      </c>
+      <c r="H1" t="s">
+        <v>595</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8">
+      <c r="A2" t="s">
+        <v>631</v>
+      </c>
+      <c r="B2">
+        <v>16</v>
+      </c>
+      <c r="C2">
+        <v>0</v>
+      </c>
+      <c r="D2">
+        <v>2</v>
+      </c>
+      <c r="E2" t="s">
+        <v>173</v>
+      </c>
+      <c r="F2" t="s">
+        <v>173</v>
+      </c>
+      <c r="G2" t="s">
+        <v>602</v>
+      </c>
+      <c r="H2">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8">
+      <c r="A3" t="s">
+        <v>631</v>
+      </c>
+      <c r="B3">
+        <v>17</v>
+      </c>
+      <c r="C3">
+        <v>0</v>
+      </c>
+      <c r="D3">
+        <v>2</v>
+      </c>
+      <c r="E3" t="s">
+        <v>79</v>
+      </c>
+      <c r="F3" t="s">
+        <v>79</v>
+      </c>
+      <c r="G3" t="s">
+        <v>603</v>
+      </c>
+      <c r="H3">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8">
+      <c r="A4" t="s">
+        <v>631</v>
+      </c>
+      <c r="B4">
+        <v>18</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+      <c r="D4">
+        <v>2</v>
+      </c>
+      <c r="E4" t="s">
+        <v>110</v>
+      </c>
+      <c r="F4" t="s">
+        <v>110</v>
+      </c>
+      <c r="G4" t="s">
+        <v>604</v>
+      </c>
+      <c r="H4">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8">
+      <c r="A5" t="s">
+        <v>631</v>
+      </c>
+      <c r="B5">
+        <v>19</v>
+      </c>
+      <c r="C5">
+        <v>0</v>
+      </c>
+      <c r="D5">
+        <v>2</v>
+      </c>
+      <c r="E5" t="s">
+        <v>73</v>
+      </c>
+      <c r="F5" t="s">
+        <v>73</v>
+      </c>
+      <c r="G5" t="s">
+        <v>605</v>
+      </c>
+      <c r="H5">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8">
+      <c r="A6" t="s">
+        <v>631</v>
+      </c>
+      <c r="B6">
+        <v>22</v>
+      </c>
+      <c r="C6">
+        <v>0</v>
+      </c>
+      <c r="D6">
+        <v>2</v>
+      </c>
+      <c r="E6" t="s">
+        <v>276</v>
+      </c>
+      <c r="F6" t="s">
+        <v>276</v>
+      </c>
+      <c r="G6" t="s">
+        <v>606</v>
+      </c>
+      <c r="H6">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8">
+      <c r="A7" t="s">
+        <v>631</v>
+      </c>
+      <c r="B7">
+        <v>23</v>
+      </c>
+      <c r="C7">
+        <v>0</v>
+      </c>
+      <c r="D7">
+        <v>2</v>
+      </c>
+      <c r="E7" t="s">
+        <v>99</v>
+      </c>
+      <c r="F7" t="s">
+        <v>99</v>
+      </c>
+      <c r="G7" t="s">
+        <v>607</v>
+      </c>
+      <c r="H7">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8">
+      <c r="A8" t="s">
+        <v>631</v>
+      </c>
+      <c r="B8">
+        <v>24</v>
+      </c>
+      <c r="C8">
+        <v>0</v>
+      </c>
+      <c r="D8">
+        <v>2</v>
+      </c>
+      <c r="E8" t="s">
+        <v>251</v>
+      </c>
+      <c r="F8" t="s">
+        <v>251</v>
+      </c>
+      <c r="G8" t="s">
+        <v>608</v>
+      </c>
+      <c r="H8">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8">
+      <c r="A9" t="s">
+        <v>631</v>
+      </c>
+      <c r="B9">
+        <v>25</v>
+      </c>
+      <c r="C9">
+        <v>0</v>
+      </c>
+      <c r="D9">
+        <v>2</v>
+      </c>
+      <c r="E9" t="s">
+        <v>100</v>
+      </c>
+      <c r="F9" t="s">
+        <v>100</v>
+      </c>
+      <c r="G9" t="s">
+        <v>609</v>
+      </c>
+      <c r="H9">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8">
+      <c r="A10" t="s">
+        <v>631</v>
+      </c>
+      <c r="B10">
+        <v>26</v>
+      </c>
+      <c r="C10">
+        <v>0</v>
+      </c>
+      <c r="D10">
+        <v>2</v>
+      </c>
+      <c r="E10" t="s">
+        <v>610</v>
+      </c>
+      <c r="F10" t="s">
+        <v>610</v>
+      </c>
+      <c r="G10" t="s">
+        <v>611</v>
+      </c>
+      <c r="H10">
+        <v>572</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8">
+      <c r="A11" t="s">
+        <v>631</v>
+      </c>
+      <c r="B11">
+        <v>27</v>
+      </c>
+      <c r="C11">
+        <v>0</v>
+      </c>
+      <c r="D11">
+        <v>2</v>
+      </c>
+      <c r="E11" t="s">
+        <v>612</v>
+      </c>
+      <c r="F11" t="s">
+        <v>613</v>
+      </c>
+      <c r="G11" t="s">
+        <v>614</v>
+      </c>
+      <c r="H11">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8">
+      <c r="A12" t="s">
+        <v>631</v>
+      </c>
+      <c r="B12">
+        <v>28</v>
+      </c>
+      <c r="C12">
+        <v>0</v>
+      </c>
+      <c r="D12">
+        <v>2</v>
+      </c>
+      <c r="E12" t="s">
+        <v>321</v>
+      </c>
+      <c r="F12" t="s">
+        <v>321</v>
+      </c>
+      <c r="G12" t="s">
+        <v>615</v>
+      </c>
+      <c r="H12">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8">
+      <c r="A13" t="s">
+        <v>631</v>
+      </c>
+      <c r="B13">
+        <v>29</v>
+      </c>
+      <c r="C13">
+        <v>0</v>
+      </c>
+      <c r="D13">
+        <v>2</v>
+      </c>
+      <c r="E13" t="s">
+        <v>616</v>
+      </c>
+      <c r="F13" t="s">
+        <v>271</v>
+      </c>
+      <c r="G13" t="s">
+        <v>617</v>
+      </c>
+      <c r="H13">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8">
+      <c r="A14" t="s">
+        <v>631</v>
+      </c>
+      <c r="B14">
+        <v>30</v>
+      </c>
+      <c r="C14">
+        <v>0</v>
+      </c>
+      <c r="D14">
+        <v>2</v>
+      </c>
+      <c r="E14" t="s">
+        <v>618</v>
+      </c>
+      <c r="F14" t="s">
+        <v>618</v>
+      </c>
+      <c r="G14" t="s">
+        <v>618</v>
+      </c>
+      <c r="H14">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8">
+      <c r="A15" t="s">
+        <v>86</v>
+      </c>
+      <c r="B15">
+        <v>31</v>
+      </c>
+      <c r="C15">
+        <v>0</v>
+      </c>
+      <c r="D15">
+        <v>2</v>
+      </c>
+      <c r="E15" t="s">
+        <v>619</v>
+      </c>
+      <c r="F15" t="s">
+        <v>619</v>
+      </c>
+      <c r="G15" t="s">
+        <v>619</v>
+      </c>
+      <c r="H15">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8">
+      <c r="A16" t="s">
+        <v>86</v>
+      </c>
+      <c r="B16">
+        <v>32</v>
+      </c>
+      <c r="C16">
+        <v>0</v>
+      </c>
+      <c r="D16">
+        <v>2</v>
+      </c>
+      <c r="E16" t="s">
+        <v>620</v>
+      </c>
+      <c r="F16" t="s">
+        <v>620</v>
+      </c>
+      <c r="G16" t="s">
+        <v>620</v>
+      </c>
+      <c r="H16">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8">
+      <c r="A17" t="s">
+        <v>87</v>
+      </c>
+      <c r="B17">
+        <v>33</v>
+      </c>
+      <c r="C17">
+        <v>0</v>
+      </c>
+      <c r="D17">
+        <v>2</v>
+      </c>
+      <c r="E17" t="s">
+        <v>621</v>
+      </c>
+      <c r="F17" t="s">
+        <v>621</v>
+      </c>
+      <c r="G17" t="s">
+        <v>621</v>
+      </c>
+      <c r="H17">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8">
+      <c r="A18" t="s">
+        <v>87</v>
+      </c>
+      <c r="B18">
+        <v>34</v>
+      </c>
+      <c r="C18">
+        <v>0</v>
+      </c>
+      <c r="D18">
+        <v>2</v>
+      </c>
+      <c r="E18" t="s">
+        <v>622</v>
+      </c>
+      <c r="F18" t="s">
+        <v>622</v>
+      </c>
+      <c r="G18" t="s">
+        <v>622</v>
+      </c>
+      <c r="H18">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8">
+      <c r="A19" t="s">
+        <v>155</v>
+      </c>
+      <c r="B19">
+        <v>35</v>
+      </c>
+      <c r="C19">
+        <v>0</v>
+      </c>
+      <c r="D19">
+        <v>2</v>
+      </c>
+      <c r="E19" t="s">
+        <v>623</v>
+      </c>
+      <c r="F19" t="s">
+        <v>623</v>
+      </c>
+      <c r="G19" t="s">
+        <v>623</v>
+      </c>
+      <c r="H19">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8">
+      <c r="A20" t="s">
+        <v>155</v>
+      </c>
+      <c r="B20">
+        <v>36</v>
+      </c>
+      <c r="C20">
+        <v>0</v>
+      </c>
+      <c r="D20">
+        <v>2</v>
+      </c>
+      <c r="E20" t="s">
+        <v>624</v>
+      </c>
+      <c r="F20" t="s">
+        <v>624</v>
+      </c>
+      <c r="G20" t="s">
+        <v>624</v>
+      </c>
+      <c r="H20">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8">
+      <c r="A21" t="s">
+        <v>631</v>
+      </c>
+      <c r="B21">
+        <v>43</v>
+      </c>
+      <c r="C21">
+        <v>0</v>
+      </c>
+      <c r="D21">
+        <v>5</v>
+      </c>
+      <c r="E21" t="s">
+        <v>625</v>
+      </c>
+      <c r="F21" t="s">
+        <v>625</v>
+      </c>
+      <c r="H21">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8">
+      <c r="A22" t="s">
+        <v>631</v>
+      </c>
+      <c r="B22">
+        <v>44</v>
+      </c>
+      <c r="C22">
+        <v>0</v>
+      </c>
+      <c r="D22">
+        <v>2</v>
+      </c>
+      <c r="E22" t="s">
+        <v>625</v>
+      </c>
+      <c r="F22" t="s">
+        <v>625</v>
+      </c>
+      <c r="G22" t="s">
+        <v>626</v>
+      </c>
+      <c r="H22">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8">
+      <c r="A23" t="s">
+        <v>631</v>
+      </c>
+      <c r="B23">
+        <v>45</v>
+      </c>
+      <c r="C23">
+        <v>0</v>
+      </c>
+      <c r="D23">
+        <v>2</v>
+      </c>
+      <c r="E23" t="s">
+        <v>627</v>
+      </c>
+      <c r="F23" t="s">
+        <v>627</v>
+      </c>
+      <c r="G23" t="s">
+        <v>628</v>
+      </c>
+      <c r="H23">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8">
+      <c r="A24" t="s">
+        <v>631</v>
+      </c>
+      <c r="B24">
+        <v>46</v>
+      </c>
+      <c r="C24">
+        <v>0</v>
+      </c>
+      <c r="D24">
+        <v>2</v>
+      </c>
+      <c r="E24" t="s">
+        <v>629</v>
+      </c>
+      <c r="F24" t="s">
+        <v>629</v>
+      </c>
+      <c r="G24" t="s">
+        <v>630</v>
+      </c>
+      <c r="H24">
+        <v>50</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:A248"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -43821,7 +44838,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:A102"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -44342,282 +45359,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G10"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="7" max="7" width="23" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:7">
-      <c r="A1" t="s">
-        <v>589</v>
-      </c>
-      <c r="B1" t="s">
-        <v>590</v>
-      </c>
-      <c r="C1" t="s">
-        <v>591</v>
-      </c>
-      <c r="D1" t="s">
-        <v>592</v>
-      </c>
-      <c r="E1" t="s">
-        <v>593</v>
-      </c>
-      <c r="F1" t="s">
-        <v>594</v>
-      </c>
-      <c r="G1" t="s">
-        <v>632</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7">
-      <c r="A2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2">
-        <v>1</v>
-      </c>
-      <c r="C2" t="str">
-        <f>IF(MID(A2,3,1)=" ",LEFT(A2,2)&amp;MID(A2,4,LEN(A2)-3),A2)</f>
-        <v>CE1202</v>
-      </c>
-      <c r="D2" t="str">
-        <f>MID(C2,4,1)</f>
-        <v>2</v>
-      </c>
-      <c r="E2" t="b">
-        <f>IF(F2="IS",TRUE,FALSE)</f>
-        <v>0</v>
-      </c>
-      <c r="F2" t="str">
-        <f>LEFT(C2,2)</f>
-        <v>CE</v>
-      </c>
-      <c r="G2">
-        <v>550</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7">
-      <c r="A3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B3">
-        <v>1</v>
-      </c>
-      <c r="C3" t="str">
-        <f t="shared" ref="C3:C10" si="0">IF(MID(A3,3,1)=" ",LEFT(A3,2)&amp;MID(A3,4,LEN(A3)-3),A3)</f>
-        <v>CE1101</v>
-      </c>
-      <c r="D3" t="str">
-        <f t="shared" ref="D3:D9" si="1">MID(C3,4,1)</f>
-        <v>1</v>
-      </c>
-      <c r="E3" t="b">
-        <f t="shared" ref="E3:E10" si="2">IF(F3="IS",TRUE,FALSE)</f>
-        <v>0</v>
-      </c>
-      <c r="F3" t="str">
-        <f t="shared" ref="F3:F10" si="3">LEFT(C3,2)</f>
-        <v>CE</v>
-      </c>
-      <c r="G3">
-        <v>550</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7">
-      <c r="A4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4">
-        <v>1</v>
-      </c>
-      <c r="C4" t="str">
-        <f t="shared" si="0"/>
-        <v>EE1301</v>
-      </c>
-      <c r="D4" t="str">
-        <f t="shared" si="1"/>
-        <v>3</v>
-      </c>
-      <c r="E4" t="b">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="F4" t="str">
-        <f t="shared" si="3"/>
-        <v>EE</v>
-      </c>
-      <c r="G4">
-        <v>550</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7">
-      <c r="A5" t="s">
-        <v>12</v>
-      </c>
-      <c r="B5">
-        <v>1</v>
-      </c>
-      <c r="C5" t="str">
-        <f t="shared" si="0"/>
-        <v>EE1101</v>
-      </c>
-      <c r="D5" t="str">
-        <f t="shared" si="1"/>
-        <v>1</v>
-      </c>
-      <c r="E5" t="b">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="F5" t="str">
-        <f t="shared" si="3"/>
-        <v>EE</v>
-      </c>
-      <c r="G5">
-        <v>550</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7">
-      <c r="A6" t="s">
-        <v>14</v>
-      </c>
-      <c r="B6">
-        <v>1</v>
-      </c>
-      <c r="C6" t="str">
-        <f t="shared" si="0"/>
-        <v>ME1201</v>
-      </c>
-      <c r="D6" t="str">
-        <f t="shared" si="1"/>
-        <v>2</v>
-      </c>
-      <c r="E6" t="b">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="F6" t="str">
-        <f t="shared" si="3"/>
-        <v>ME</v>
-      </c>
-      <c r="G6">
-        <v>550</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7">
-      <c r="A7" t="s">
-        <v>16</v>
-      </c>
-      <c r="B7">
-        <v>1</v>
-      </c>
-      <c r="C7" t="str">
-        <f t="shared" si="0"/>
-        <v>ME1202</v>
-      </c>
-      <c r="D7" t="str">
-        <f t="shared" si="1"/>
-        <v>2</v>
-      </c>
-      <c r="E7" t="b">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="F7" t="str">
-        <f t="shared" si="3"/>
-        <v>ME</v>
-      </c>
-      <c r="G7">
-        <v>550</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7">
-      <c r="A8" t="s">
-        <v>18</v>
-      </c>
-      <c r="B8">
-        <v>1</v>
-      </c>
-      <c r="C8" t="str">
-        <f t="shared" si="0"/>
-        <v>IS1402</v>
-      </c>
-      <c r="D8" t="str">
-        <f t="shared" si="1"/>
-        <v>4</v>
-      </c>
-      <c r="E8" t="b">
-        <f t="shared" si="2"/>
-        <v>1</v>
-      </c>
-      <c r="F8" t="str">
-        <f t="shared" si="3"/>
-        <v>IS</v>
-      </c>
-      <c r="G8">
-        <v>550</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7">
-      <c r="A9" t="s">
-        <v>20</v>
-      </c>
-      <c r="B9">
-        <v>1</v>
-      </c>
-      <c r="C9" t="str">
-        <f t="shared" si="0"/>
-        <v>IS1301</v>
-      </c>
-      <c r="D9" t="str">
-        <f t="shared" si="1"/>
-        <v>3</v>
-      </c>
-      <c r="E9" t="b">
-        <f t="shared" si="2"/>
-        <v>1</v>
-      </c>
-      <c r="F9" t="str">
-        <f t="shared" si="3"/>
-        <v>IS</v>
-      </c>
-      <c r="G9">
-        <v>550</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7">
-      <c r="A10" t="s">
-        <v>22</v>
-      </c>
-      <c r="B10">
-        <v>1</v>
-      </c>
-      <c r="C10" t="str">
-        <f t="shared" si="0"/>
-        <v>IS1003</v>
-      </c>
-      <c r="D10">
-        <v>2</v>
-      </c>
-      <c r="E10" t="b">
-        <f t="shared" si="2"/>
-        <v>1</v>
-      </c>
-      <c r="F10" t="str">
-        <f t="shared" si="3"/>
-        <v>IS</v>
-      </c>
-      <c r="G10">
-        <v>550</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>